<commit_message>
Update Six Sigma rating column to Dat chuan instead of Xuat sac in Excel and Word
</commit_message>
<xml_diff>
--- a/public/Bang_Du_Lieu_QC_T8_T9_2026.xlsx
+++ b/public/Bang_Du_Lieu_QC_T8_T9_2026.xlsx
@@ -725,7 +725,7 @@
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>3.13σ (Đạt chuẩn)</t>
+          <t>3.13σ (Đạt)</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>3.15σ (Đạt chuẩn)</t>
+          <t>3.15σ (Đạt)</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>4.19σ (Mức Tốt)</t>
+          <t>4.19σ (Đạt)</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>4.30σ (Mức Tốt)</t>
+          <t>4.30σ (Đạt)</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>5.57σ (Xuất sắc)</t>
+          <t>5.57σ (Đạt)</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>5.65σ (Xuất sắc)</t>
+          <t>5.65σ (Đạt)</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>Đạt chuẩn, Tốt và Xuất sắc (3.13σ đến 5.65σ)</t>
+          <t>100% Đạt yêu cầu (3.13σ đến 5.65σ ≥ 3.0σ)</t>
         </is>
       </c>
       <c r="D9" s="21" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="E9" s="22" t="inlineStr">
         <is>
-          <t>Nâng cấp chất lượng phòng xét nghiệm lên chuẩn quốc tế</t>
+          <t>Nâng cấp chất lượng phòng xét nghiệm đạt chuẩn quy định</t>
         </is>
       </c>
     </row>

</xml_diff>